<commit_message>
8937: update unit tests
</commit_message>
<xml_diff>
--- a/shared/src/test/mockTermSpreadsheet.xlsx
+++ b/shared/src/test/mockTermSpreadsheet.xlsx
@@ -874,7 +874,7 @@
     <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -892,7 +892,7 @@
       <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -904,7 +904,7 @@
       <c r="H2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="J2" s="3" t="s">
@@ -5424,7 +5424,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5558,7 +5558,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5595,6 +5595,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>